<commit_message>
cluster analysis factoriescap_r (costs_r)
</commit_message>
<xml_diff>
--- a/clustering/8 subclusters (VDS_r (costs_r) 0 prop IQR).xlsx
+++ b/clustering/8 subclusters (VDS_r (costs_r) 0 prop IQR).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
   <si>
     <t>clust</t>
   </si>
@@ -34,9 +34,6 @@
   </si>
   <si>
     <t>trainingcosts_r</t>
-  </si>
-  <si>
-    <t>factoriescap_s</t>
   </si>
   <si>
     <t>ITcosts_s</t>
@@ -64,6 +61,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>
@@ -665,17 +664,17 @@
       <c r="A12" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update 8 subclusters (VDS_r (costs_r) 0 prop IQR).xlsx
</commit_message>
<xml_diff>
--- a/clustering/8 subclusters (VDS_r (costs_r) 0 prop IQR).xlsx
+++ b/clustering/8 subclusters (VDS_r (costs_r) 0 prop IQR).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="5">
   <si>
     <t>clust</t>
   </si>
@@ -34,15 +34,6 @@
   </si>
   <si>
     <t>trainingcosts_r</t>
-  </si>
-  <si>
-    <t>ITcosts_s</t>
-  </si>
-  <si>
-    <t>skvozcosts_s</t>
-  </si>
-  <si>
-    <t>trainingcosts_s</t>
   </si>
 </sst>
 </file>
@@ -667,14 +658,14 @@
       <c r="B12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>7</v>
+      <c r="C12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>